<commit_message>
Revised files using EPE data : BECF, BTaDLP, CCaCM, EIaE, SYC
</commit_message>
<xml_diff>
--- a/InputData/elec/BTaDLP/BAU Trans and Distr Loss Perc.xlsx
+++ b/InputData/elec/BTaDLP/BAU Trans and Distr Loss Perc.xlsx
@@ -1,23 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27425"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="14420"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\shigu\Documents\_swj\_Talanoa\CPSA Fletcher\dados\InputData (BR) 2024\d08 elec\BTaDLP\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\saido\Documents\eps-brazil-cpl\InputData\elec\BTaDLP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F88FE615-B3E6-4299-8B8C-472CDDEE6E62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="168" yWindow="492" windowWidth="22728" windowHeight="11004" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="165" yWindow="495" windowWidth="22725" windowHeight="11010" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
     <sheet name="Calculations" sheetId="4" r:id="rId2"/>
     <sheet name="BTaDLP" sheetId="2" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="152511"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -34,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="29">
   <si>
     <t>BTaDLP BAU Transmission and Distribution Loss Percentage</t>
   </si>
@@ -106,12 +105,27 @@
   </si>
   <si>
     <t>at the average value the period 2016-2022.</t>
+  </si>
+  <si>
+    <t>Metric / Year</t>
+  </si>
+  <si>
+    <t>average</t>
+  </si>
+  <si>
+    <t>Production (GWh)</t>
+  </si>
+  <si>
+    <t>Losses  (GWh)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Losses  </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.000"/>
   </numFmts>
@@ -198,7 +212,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -235,12 +249,28 @@
     <xf numFmtId="10" fontId="6" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="4">
-    <cellStyle name="Hiperlink" xfId="1" builtinId="8"/>
+    <cellStyle name="Lien hypertexte" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 2" xfId="2" xr:uid="{00000000-0005-0000-0000-000002000000}"/>
-    <cellStyle name="Porcentagem" xfId="3" builtinId="5"/>
+    <cellStyle name="Normal 2" xfId="2"/>
+    <cellStyle name="Pourcentage" xfId="3" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -265,8 +295,8 @@
       <xdr:rowOff>160020</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>17</xdr:col>
-      <xdr:colOff>5823</xdr:colOff>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>320148</xdr:colOff>
       <xdr:row>28</xdr:row>
       <xdr:rowOff>160020</xdr:rowOff>
     </xdr:to>
@@ -275,7 +305,7 @@
         <xdr:cNvPr id="4" name="Imagem 3">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{BCBE3086-7CC8-C43D-AEB3-D4C416D25E8E}"/>
+              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{BCBE3086-7CC8-C43D-AEB3-D4C416D25E8E}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -319,7 +349,7 @@
         <xdr:cNvPr id="5" name="Imagem 4">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{25FDA29C-FDE5-4C65-A801-7C6AE64DA440}"/>
+              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{25FDA29C-FDE5-4C65-A801-7C6AE64DA440}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -349,9 +379,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Thème Office">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -389,9 +419,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -426,7 +456,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -461,7 +491,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -634,23 +664,23 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="63.77734375" customWidth="1"/>
-    <col min="3" max="3" width="8.88671875" style="8"/>
+    <col min="2" max="2" width="63.7109375" customWidth="1"/>
+    <col min="3" max="3" width="8.85546875" style="8"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="1"/>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>6</v>
       </c>
@@ -661,7 +691,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
       <c r="B4" t="s">
         <v>9</v>
@@ -670,54 +700,54 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
       <c r="B5" s="2">
         <v>2022</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
       <c r="B6" s="3" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="10" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>20</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="B6" r:id="rId1" location="!" xr:uid="{58F9F47D-E2FD-4C16-A0A3-C9189CF90A28}"/>
+    <hyperlink ref="B6" r:id="rId1" location="!"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId2"/>
@@ -725,17 +755,20 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:F28"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:K35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.44140625" customWidth="1"/>
-    <col min="2" max="2" width="9.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.33203125" customWidth="1"/>
+    <col min="1" max="1" width="33" customWidth="1"/>
+    <col min="2" max="2" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.28515625" customWidth="1"/>
     <col min="4" max="4" width="12" customWidth="1"/>
+    <col min="5" max="7" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="9" max="11" width="11.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="11"/>
       <c r="B1" s="12" t="s">
         <v>16</v>
@@ -747,7 +780,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="12">
         <v>2008</v>
       </c>
@@ -766,7 +799,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="12">
         <v>2009</v>
       </c>
@@ -783,7 +816,7 @@
       <c r="E3" s="13"/>
       <c r="F3" s="13"/>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="12">
         <v>2010</v>
       </c>
@@ -800,7 +833,7 @@
       <c r="E4" s="13"/>
       <c r="F4" s="13"/>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="12">
         <v>2011</v>
       </c>
@@ -816,7 +849,7 @@
       </c>
       <c r="E5" s="13"/>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="12">
         <v>2012</v>
       </c>
@@ -833,7 +866,7 @@
       <c r="E6" s="13"/>
       <c r="F6" s="13"/>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="12">
         <v>2013</v>
       </c>
@@ -850,7 +883,7 @@
       <c r="E7" s="13"/>
       <c r="F7" s="13"/>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="12">
         <v>2014</v>
       </c>
@@ -867,7 +900,7 @@
       <c r="E8" s="13"/>
       <c r="F8" s="13"/>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="12">
         <v>2015</v>
       </c>
@@ -884,7 +917,7 @@
       <c r="E9" s="13"/>
       <c r="F9" s="13"/>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="12">
         <v>2016</v>
       </c>
@@ -901,7 +934,7 @@
       <c r="E10" s="13"/>
       <c r="F10" s="13"/>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="12">
         <v>2017</v>
       </c>
@@ -918,7 +951,7 @@
       <c r="E11" s="13"/>
       <c r="F11" s="13"/>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="12">
         <v>2018</v>
       </c>
@@ -935,7 +968,7 @@
       <c r="E12" s="13"/>
       <c r="F12" s="13"/>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="12">
         <v>2019</v>
       </c>
@@ -952,7 +985,7 @@
       <c r="E13" s="13"/>
       <c r="F13" s="13"/>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="12">
         <v>2020</v>
       </c>
@@ -969,7 +1002,7 @@
       <c r="E14" s="13"/>
       <c r="F14" s="13"/>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="12">
         <v>2021</v>
       </c>
@@ -986,7 +1019,7 @@
       <c r="E15" s="13"/>
       <c r="F15" s="13"/>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="12">
         <v>2022</v>
       </c>
@@ -1003,7 +1036,7 @@
       <c r="E16" s="13"/>
       <c r="F16" s="13"/>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" s="18" t="s">
         <v>21</v>
       </c>
@@ -1014,12 +1047,12 @@
       <c r="C17" s="5"/>
       <c r="D17" s="4"/>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B18" s="5"/>
       <c r="C18" s="5"/>
       <c r="D18" s="4"/>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" s="16" t="s">
         <v>22</v>
       </c>
@@ -1027,7 +1060,7 @@
       <c r="C19" s="5"/>
       <c r="D19" s="4"/>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" s="10" t="s">
         <v>23</v>
       </c>
@@ -1035,36 +1068,36 @@
       <c r="C20" s="5"/>
       <c r="D20" s="4"/>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" s="1"/>
       <c r="B21" s="5"/>
       <c r="C21" s="5"/>
       <c r="D21" s="4"/>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" s="1"/>
       <c r="B22" s="5"/>
       <c r="C22" s="5"/>
       <c r="D22" s="4"/>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" s="1"/>
       <c r="B23" s="5"/>
       <c r="C23" s="5"/>
       <c r="D23" s="4"/>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" s="1"/>
       <c r="B24" s="5"/>
       <c r="C24" s="5"/>
       <c r="D24" s="4"/>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
         <v>2</v>
       </c>
@@ -1073,6 +1106,165 @@
       <c r="D28" s="6">
         <f>AVERAGE(D2:D23)</f>
         <v>0.13868000000000003</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="21" t="s">
+        <v>24</v>
+      </c>
+      <c r="B31" s="22">
+        <v>2015</v>
+      </c>
+      <c r="C31" s="22">
+        <v>2016</v>
+      </c>
+      <c r="D31" s="22">
+        <v>2017</v>
+      </c>
+      <c r="E31" s="22">
+        <v>2018</v>
+      </c>
+      <c r="F31" s="22">
+        <v>2019</v>
+      </c>
+      <c r="G31" s="22">
+        <v>2020</v>
+      </c>
+      <c r="H31" s="22">
+        <v>2021</v>
+      </c>
+      <c r="I31" s="22">
+        <v>2022</v>
+      </c>
+      <c r="J31" s="22">
+        <v>2023</v>
+      </c>
+      <c r="K31" s="22">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A32" s="20" t="s">
+        <v>26</v>
+      </c>
+      <c r="B32" s="23">
+        <v>586647</v>
+      </c>
+      <c r="C32" s="23">
+        <v>584388</v>
+      </c>
+      <c r="D32" s="23">
+        <v>595574</v>
+      </c>
+      <c r="E32" s="23">
+        <v>607203</v>
+      </c>
+      <c r="F32" s="23">
+        <v>633032</v>
+      </c>
+      <c r="G32" s="23">
+        <v>628764</v>
+      </c>
+      <c r="H32" s="23">
+        <v>656396</v>
+      </c>
+      <c r="I32" s="23">
+        <v>677162</v>
+      </c>
+      <c r="J32" s="23">
+        <v>708119</v>
+      </c>
+      <c r="K32" s="23">
+        <v>751335</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A33" s="20" t="s">
+        <v>27</v>
+      </c>
+      <c r="B33" s="23">
+        <v>90901</v>
+      </c>
+      <c r="C33" s="23">
+        <v>98317</v>
+      </c>
+      <c r="D33" s="23">
+        <v>97619</v>
+      </c>
+      <c r="E33" s="23">
+        <v>97973</v>
+      </c>
+      <c r="F33" s="23">
+        <v>105912</v>
+      </c>
+      <c r="G33" s="23">
+        <v>105766</v>
+      </c>
+      <c r="H33" s="23">
+        <v>106348</v>
+      </c>
+      <c r="I33" s="23">
+        <v>103995</v>
+      </c>
+      <c r="J33" s="23">
+        <v>106919</v>
+      </c>
+      <c r="K33" s="23">
+        <v>112492</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A34" s="20" t="s">
+        <v>28</v>
+      </c>
+      <c r="B34" s="24">
+        <f>B33/B32</f>
+        <v>0.15495008071293298</v>
+      </c>
+      <c r="C34" s="24">
+        <f t="shared" ref="C34:K34" si="1">C33/C32</f>
+        <v>0.16823925200380568</v>
+      </c>
+      <c r="D34" s="24">
+        <f t="shared" si="1"/>
+        <v>0.16390742376262227</v>
+      </c>
+      <c r="E34" s="24">
+        <f t="shared" si="1"/>
+        <v>0.16135131084661966</v>
+      </c>
+      <c r="F34" s="24">
+        <f t="shared" si="1"/>
+        <v>0.16730907758217595</v>
+      </c>
+      <c r="G34" s="24">
+        <f t="shared" si="1"/>
+        <v>0.16821255669853871</v>
+      </c>
+      <c r="H34" s="24">
+        <f t="shared" si="1"/>
+        <v>0.16201805007952516</v>
+      </c>
+      <c r="I34" s="24">
+        <f t="shared" si="1"/>
+        <v>0.15357477235875611</v>
+      </c>
+      <c r="J34" s="24">
+        <f t="shared" si="1"/>
+        <v>0.15099015843382257</v>
+      </c>
+      <c r="K34" s="24">
+        <f t="shared" si="1"/>
+        <v>0.14972282670180412</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A35" s="20" t="s">
+        <v>25</v>
+      </c>
+      <c r="B35" s="25">
+        <f>ROUND(AVERAGE(B34:K34),3)</f>
+        <v>0.16</v>
       </c>
     </row>
   </sheetData>
@@ -1083,18 +1275,18 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:AK2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="20.44140625" customWidth="1"/>
+    <col min="1" max="1" width="20.42578125" customWidth="1"/>
     <col min="2" max="2" width="9" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:37" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>3</v>
       </c>
@@ -1207,145 +1399,153 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="2" spans="1:37" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:37" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
         <v>5</v>
       </c>
       <c r="B2" s="4">
-        <v>7.400000000000001E-2</v>
-      </c>
-      <c r="C2" s="4">
-        <v>7.4900000000000008E-2</v>
-      </c>
-      <c r="D2" s="4">
-        <v>7.46E-2</v>
-      </c>
-      <c r="E2" s="4">
-        <v>7.4299999999999991E-2</v>
-      </c>
-      <c r="F2" s="4">
-        <v>7.4099999999999999E-2</v>
-      </c>
-      <c r="G2" s="4">
-        <v>7.4099999999999999E-2</v>
-      </c>
-      <c r="H2" s="4">
-        <v>7.3800000000000004E-2</v>
-      </c>
-      <c r="I2" s="4">
-        <v>7.3800000000000004E-2</v>
-      </c>
-      <c r="J2" s="4">
-        <f>Calculations!B17</f>
-        <v>7.4228571428571422E-2</v>
-      </c>
-      <c r="K2" s="4">
-        <f>$J2</f>
-        <v>7.4228571428571422E-2</v>
+        <f>Calculations!B35</f>
+        <v>0.16</v>
+      </c>
+      <c r="C2" s="17">
+        <f>B2</f>
+        <v>0.16</v>
+      </c>
+      <c r="D2" s="17">
+        <f t="shared" ref="D2:AK2" si="0">C2</f>
+        <v>0.16</v>
+      </c>
+      <c r="E2" s="17">
+        <f t="shared" si="0"/>
+        <v>0.16</v>
+      </c>
+      <c r="F2" s="17">
+        <f t="shared" si="0"/>
+        <v>0.16</v>
+      </c>
+      <c r="G2" s="17">
+        <f t="shared" si="0"/>
+        <v>0.16</v>
+      </c>
+      <c r="H2" s="17">
+        <f t="shared" si="0"/>
+        <v>0.16</v>
+      </c>
+      <c r="I2" s="17">
+        <f t="shared" si="0"/>
+        <v>0.16</v>
+      </c>
+      <c r="J2" s="17">
+        <f t="shared" si="0"/>
+        <v>0.16</v>
+      </c>
+      <c r="K2" s="17">
+        <f t="shared" si="0"/>
+        <v>0.16</v>
       </c>
       <c r="L2" s="17">
-        <f t="shared" ref="L2:AK2" si="0">$J2</f>
-        <v>7.4228571428571422E-2</v>
+        <f t="shared" si="0"/>
+        <v>0.16</v>
       </c>
       <c r="M2" s="17">
         <f t="shared" si="0"/>
-        <v>7.4228571428571422E-2</v>
+        <v>0.16</v>
       </c>
       <c r="N2" s="17">
         <f t="shared" si="0"/>
-        <v>7.4228571428571422E-2</v>
+        <v>0.16</v>
       </c>
       <c r="O2" s="17">
         <f t="shared" si="0"/>
-        <v>7.4228571428571422E-2</v>
+        <v>0.16</v>
       </c>
       <c r="P2" s="17">
         <f t="shared" si="0"/>
-        <v>7.4228571428571422E-2</v>
+        <v>0.16</v>
       </c>
       <c r="Q2" s="17">
         <f t="shared" si="0"/>
-        <v>7.4228571428571422E-2</v>
+        <v>0.16</v>
       </c>
       <c r="R2" s="17">
         <f t="shared" si="0"/>
-        <v>7.4228571428571422E-2</v>
+        <v>0.16</v>
       </c>
       <c r="S2" s="17">
         <f t="shared" si="0"/>
-        <v>7.4228571428571422E-2</v>
+        <v>0.16</v>
       </c>
       <c r="T2" s="17">
         <f t="shared" si="0"/>
-        <v>7.4228571428571422E-2</v>
+        <v>0.16</v>
       </c>
       <c r="U2" s="17">
         <f t="shared" si="0"/>
-        <v>7.4228571428571422E-2</v>
+        <v>0.16</v>
       </c>
       <c r="V2" s="17">
         <f t="shared" si="0"/>
-        <v>7.4228571428571422E-2</v>
+        <v>0.16</v>
       </c>
       <c r="W2" s="17">
         <f t="shared" si="0"/>
-        <v>7.4228571428571422E-2</v>
+        <v>0.16</v>
       </c>
       <c r="X2" s="17">
         <f t="shared" si="0"/>
-        <v>7.4228571428571422E-2</v>
+        <v>0.16</v>
       </c>
       <c r="Y2" s="17">
         <f t="shared" si="0"/>
-        <v>7.4228571428571422E-2</v>
+        <v>0.16</v>
       </c>
       <c r="Z2" s="17">
         <f t="shared" si="0"/>
-        <v>7.4228571428571422E-2</v>
+        <v>0.16</v>
       </c>
       <c r="AA2" s="17">
         <f t="shared" si="0"/>
-        <v>7.4228571428571422E-2</v>
+        <v>0.16</v>
       </c>
       <c r="AB2" s="17">
         <f t="shared" si="0"/>
-        <v>7.4228571428571422E-2</v>
+        <v>0.16</v>
       </c>
       <c r="AC2" s="17">
         <f t="shared" si="0"/>
-        <v>7.4228571428571422E-2</v>
+        <v>0.16</v>
       </c>
       <c r="AD2" s="17">
         <f t="shared" si="0"/>
-        <v>7.4228571428571422E-2</v>
+        <v>0.16</v>
       </c>
       <c r="AE2" s="17">
         <f t="shared" si="0"/>
-        <v>7.4228571428571422E-2</v>
+        <v>0.16</v>
       </c>
       <c r="AF2" s="17">
         <f t="shared" si="0"/>
-        <v>7.4228571428571422E-2</v>
+        <v>0.16</v>
       </c>
       <c r="AG2" s="17">
         <f t="shared" si="0"/>
-        <v>7.4228571428571422E-2</v>
+        <v>0.16</v>
       </c>
       <c r="AH2" s="17">
         <f t="shared" si="0"/>
-        <v>7.4228571428571422E-2</v>
+        <v>0.16</v>
       </c>
       <c r="AI2" s="17">
         <f t="shared" si="0"/>
-        <v>7.4228571428571422E-2</v>
+        <v>0.16</v>
       </c>
       <c r="AJ2" s="17">
         <f t="shared" si="0"/>
-        <v>7.4228571428571422E-2</v>
+        <v>0.16</v>
       </c>
       <c r="AK2" s="17">
         <f t="shared" si="0"/>
-        <v>7.4228571428571422E-2</v>
+        <v>0.16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>